<commit_message>
GAP-013: rider returns wait for the goods at the shop; GAP-019: fewer sequential reads in checkout and a slow-checkout timing log
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DwaGzMfLXpSfXKxyFUVJ2D
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-25.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-25.xlsx
@@ -971,7 +971,7 @@
     <row r="3" ht="24" customFormat="1" customHeight="1" s="37">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Baseline = the 24 Oct status report. Change since then: GAP-008 (map Confirm location) BLOCKED -&gt; COMPLETED, no code change.</t>
+          <t>Baseline = the 24 Oct status report. Changes since then: GAP-008 BLOCKED -&gt; COMPLETED (no code change); GAP-013 COMPLETED and GAP-019 IN PROGRESS (open PR).</t>
         </is>
       </c>
     </row>
@@ -30214,7 +30214,7 @@
       </c>
       <c r="F262" s="69" t="inlineStr">
         <is>
-          <t>Manual completion of a return pickup is offered to staff only once a rider is on the way.</t>
+          <t>Staff cannot complete a return pickup by hand while the rider has not brought the goods back. Owner decision 25 Oct: staff wait for the rider to return the goods to the shop, then press 'Goods received' to complete. The return page now tells the shop and support to wait.</t>
         </is>
       </c>
       <c r="G262" s="69" t="inlineStr">
@@ -30229,52 +30229,52 @@
       </c>
       <c r="I262" s="52" t="inlineStr">
         <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="J262" s="69" t="inlineStr">
+        <is>
+          <t>Open PR - not merged</t>
+        </is>
+      </c>
+      <c r="K262" s="69" t="inlineStr">
+        <is>
+          <t>Live once released (no switch)</t>
+        </is>
+      </c>
+      <c r="L262" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M262" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N262" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O262" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P262" s="69" t="inlineStr">
+        <is>
           <t>YET TO START</t>
         </is>
       </c>
-      <c r="J262" s="69" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K262" s="69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L262" s="69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M262" s="69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N262" s="69" t="inlineStr">
-        <is>
-          <t>Decide whether staff may complete a pickup without a rider</t>
-        </is>
-      </c>
-      <c r="O262" s="69" t="inlineStr">
-        <is>
-          <t>Owner: business rule</t>
-        </is>
-      </c>
-      <c r="P262" s="69" t="inlineStr">
-        <is>
-          <t>YET TO START</t>
-        </is>
-      </c>
       <c r="Q262" s="69" t="inlineStr">
         <is>
-          <t>No change</t>
+          <t>YET TO START -&gt; COMPLETED (25 Oct): rule decided; waiting-for-rider notice added</t>
         </is>
       </c>
       <c r="R262" s="69" t="inlineStr">
         <is>
-          <t>GoKesari_UI_Issue_Register_2026-10-09.xlsx (TST-02)</t>
+          <t>src/server/services/returns.ts (awaitingRider); src/components/return-case.tsx; tests/integration/returns-route.test.ts</t>
         </is>
       </c>
     </row>
@@ -30769,52 +30769,52 @@
       </c>
       <c r="I268" s="52" t="inlineStr">
         <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="J268" s="69" t="inlineStr">
+        <is>
+          <t>Open PR - not merged</t>
+        </is>
+      </c>
+      <c r="K268" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L268" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M268" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N268" s="69" t="inlineStr">
+        <is>
+          <t>Checkout reads that do not depend on each other now run together, the cart shops are read once, and a slow checkout logs where its time went (CHECKOUT_SLOW_LOG_MS, default 5000). The rest of the delay is the far database (GAP-010).</t>
+        </is>
+      </c>
+      <c r="O268" s="69" t="inlineStr">
+        <is>
+          <t>Owner: GAP-010 hosting decision; then re-time wallet checkout on test</t>
+        </is>
+      </c>
+      <c r="P268" s="69" t="inlineStr">
+        <is>
           <t>YET TO START</t>
         </is>
       </c>
-      <c r="J268" s="69" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K268" s="69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L268" s="69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M268" s="69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N268" s="69" t="inlineStr">
-        <is>
-          <t>Profile checkout on test; likely the far database (GAP-010)</t>
-        </is>
-      </c>
-      <c r="O268" s="69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P268" s="69" t="inlineStr">
-        <is>
-          <t>YET TO START</t>
-        </is>
-      </c>
       <c r="Q268" s="69" t="inlineStr">
         <is>
-          <t>No change</t>
+          <t>YET TO START -&gt; IN PROGRESS (25 Oct): fewer sequential database calls</t>
         </is>
       </c>
       <c r="R268" s="69" t="inlineStr">
         <is>
-          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+          <t>src/server/services/orders.ts (checkout)</t>
         </is>
       </c>
     </row>

</xml_diff>